<commit_message>
MAJ-modèle logique (#128) b355463e157b4124438937cc4ec0ea456454799a
</commit_message>
<xml_diff>
--- a/fusionModeleLogique/ig/StructureDefinition-fr-lm-acte-imagerie.xlsx
+++ b/fusionModeleLogique/ig/StructureDefinition-fr-lm-acte-imagerie.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="569" uniqueCount="132">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-04-24T08:27:00+00:00</t>
+    <t>2026-04-24T08:33:22+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -292,13 +292,74 @@
     <t>fr-lm-section.blocNarratif</t>
   </si>
   <si>
-    <t>fr-lm-acte-imagerie.sousSection</t>
+    <t>fr-lm-acte-imagerie.author[x]</t>
   </si>
   <si>
     <t xml:space="preserve">Base
 </t>
   </si>
   <si>
+    <t>author[x] peut correspondre soit à un professionnel, soit à une organisation, soit à un système.</t>
+  </si>
+  <si>
+    <t>fr-lm-section.author[x]</t>
+  </si>
+  <si>
+    <t>fr-lm-acte-imagerie.author[x].authorProfessional</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-lm-health-professional
+</t>
+  </si>
+  <si>
+    <t>L'auteur est un professionnel de santé</t>
+  </si>
+  <si>
+    <t>fr-lm-section.author[x].authorProfessional</t>
+  </si>
+  <si>
+    <t>fr-lm-acte-imagerie.author[x].authorOrganisation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-lm-organisation
+</t>
+  </si>
+  <si>
+    <t>L'auteur est une organisation</t>
+  </si>
+  <si>
+    <t>fr-lm-section.author[x].authorOrganisation</t>
+  </si>
+  <si>
+    <t>fr-lm-acte-imagerie.author[x].authorDevice</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-lm-device
+</t>
+  </si>
+  <si>
+    <t>L'auteur est un système</t>
+  </si>
+  <si>
+    <t>fr-lm-section.author[x].authorDevice</t>
+  </si>
+  <si>
+    <t>fr-lm-acte-imagerie.informant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-lm-informant
+</t>
+  </si>
+  <si>
+    <t>Informateur</t>
+  </si>
+  <si>
+    <t>fr-lm-section.informant</t>
+  </si>
+  <si>
+    <t>fr-lm-acte-imagerie.sousSection</t>
+  </si>
+  <si>
     <t>Sous-sections</t>
   </si>
   <si>
@@ -357,7 +418,7 @@
     <t>fr-lm-acte-imagerie.entree.administrationProduits</t>
   </si>
   <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-lm-administration-produit-de-sante
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-lm-dicom-medication-administration
 </t>
   </si>
   <si>
@@ -663,7 +724,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AJ12"/>
+  <dimension ref="A1:AJ17"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="43.77734375" customWidth="true" bestFit="true"/>
@@ -676,7 +737,7 @@
     <col min="8" max="8" width="13.953125" customWidth="true" bestFit="true"/>
     <col min="9" max="9" width="11.3671875" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="83.87109375" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="84.88671875" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>
@@ -1341,13 +1402,13 @@
         <v>73</v>
       </c>
       <c r="K7" t="s" s="2">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="L7" t="s" s="2">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="M7" t="s" s="2">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
@@ -1398,7 +1459,7 @@
         <v>73</v>
       </c>
       <c r="AF7" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AG7" t="s" s="2">
         <v>74</v>
@@ -1415,10 +1476,10 @@
     </row>
     <row r="8">
       <c r="A8" t="s" s="2">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B8" t="s" s="2">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" t="s" s="2">
@@ -1429,7 +1490,7 @@
         <v>74</v>
       </c>
       <c r="G8" t="s" s="2">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="H8" t="s" s="2">
         <v>73</v>
@@ -1441,13 +1502,13 @@
         <v>73</v>
       </c>
       <c r="K8" t="s" s="2">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L8" t="s" s="2">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M8" t="s" s="2">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="N8" s="2"/>
       <c r="O8" s="2"/>
@@ -1498,13 +1559,13 @@
         <v>73</v>
       </c>
       <c r="AF8" t="s" s="2">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="AG8" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AH8" t="s" s="2">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="AI8" t="s" s="2">
         <v>73</v>
@@ -1515,10 +1576,10 @@
     </row>
     <row r="9">
       <c r="A9" t="s" s="2">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B9" t="s" s="2">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" t="s" s="2">
@@ -1529,7 +1590,7 @@
         <v>74</v>
       </c>
       <c r="G9" t="s" s="2">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="H9" t="s" s="2">
         <v>73</v>
@@ -1541,13 +1602,13 @@
         <v>73</v>
       </c>
       <c r="K9" t="s" s="2">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="L9" t="s" s="2">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="M9" t="s" s="2">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="N9" s="2"/>
       <c r="O9" s="2"/>
@@ -1598,13 +1659,13 @@
         <v>73</v>
       </c>
       <c r="AF9" t="s" s="2">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="AG9" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AH9" t="s" s="2">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="AI9" t="s" s="2">
         <v>73</v>
@@ -1615,10 +1676,10 @@
     </row>
     <row r="10">
       <c r="A10" t="s" s="2">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="B10" t="s" s="2">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" t="s" s="2">
@@ -1626,10 +1687,10 @@
       </c>
       <c r="E10" s="2"/>
       <c r="F10" t="s" s="2">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="G10" t="s" s="2">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="H10" t="s" s="2">
         <v>73</v>
@@ -1641,13 +1702,13 @@
         <v>73</v>
       </c>
       <c r="K10" t="s" s="2">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="L10" t="s" s="2">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="M10" t="s" s="2">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="N10" s="2"/>
       <c r="O10" s="2"/>
@@ -1698,13 +1759,13 @@
         <v>73</v>
       </c>
       <c r="AF10" t="s" s="2">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="AG10" t="s" s="2">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="AH10" t="s" s="2">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="AI10" t="s" s="2">
         <v>73</v>
@@ -1715,10 +1776,10 @@
     </row>
     <row r="11">
       <c r="A11" t="s" s="2">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="B11" t="s" s="2">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" t="s" s="2">
@@ -1726,10 +1787,10 @@
       </c>
       <c r="E11" s="2"/>
       <c r="F11" t="s" s="2">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="G11" t="s" s="2">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="H11" t="s" s="2">
         <v>73</v>
@@ -1741,13 +1802,13 @@
         <v>73</v>
       </c>
       <c r="K11" t="s" s="2">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="L11" t="s" s="2">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="M11" t="s" s="2">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="N11" s="2"/>
       <c r="O11" s="2"/>
@@ -1798,13 +1859,13 @@
         <v>73</v>
       </c>
       <c r="AF11" t="s" s="2">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="AG11" t="s" s="2">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="AH11" t="s" s="2">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="AI11" t="s" s="2">
         <v>73</v>
@@ -1815,10 +1876,10 @@
     </row>
     <row r="12">
       <c r="A12" t="s" s="2">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="B12" t="s" s="2">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" t="s" s="2">
@@ -1841,13 +1902,13 @@
         <v>73</v>
       </c>
       <c r="K12" t="s" s="2">
-        <v>111</v>
+        <v>92</v>
       </c>
       <c r="L12" t="s" s="2">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="M12" t="s" s="2">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="N12" s="2"/>
       <c r="O12" s="2"/>
@@ -1898,7 +1959,7 @@
         <v>73</v>
       </c>
       <c r="AF12" t="s" s="2">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="AG12" t="s" s="2">
         <v>74</v>
@@ -1910,6 +1971,506 @@
         <v>73</v>
       </c>
       <c r="AJ12" t="s" s="2">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s" s="2">
+        <v>117</v>
+      </c>
+      <c r="B13" t="s" s="2">
+        <v>117</v>
+      </c>
+      <c r="C13" s="2"/>
+      <c r="D13" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="E13" s="2"/>
+      <c r="F13" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="G13" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="H13" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="I13" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="J13" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="K13" t="s" s="2">
+        <v>118</v>
+      </c>
+      <c r="L13" t="s" s="2">
+        <v>119</v>
+      </c>
+      <c r="M13" t="s" s="2">
+        <v>119</v>
+      </c>
+      <c r="N13" s="2"/>
+      <c r="O13" s="2"/>
+      <c r="P13" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Q13" s="2"/>
+      <c r="R13" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="S13" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="T13" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="U13" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="V13" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="W13" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="X13" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Y13" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Z13" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AA13" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AB13" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AC13" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AD13" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AE13" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AF13" t="s" s="2">
+        <v>117</v>
+      </c>
+      <c r="AG13" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AH13" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AI13" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AJ13" t="s" s="2">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s" s="2">
+        <v>120</v>
+      </c>
+      <c r="B14" t="s" s="2">
+        <v>120</v>
+      </c>
+      <c r="C14" s="2"/>
+      <c r="D14" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="E14" s="2"/>
+      <c r="F14" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="G14" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="H14" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="I14" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="J14" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="K14" t="s" s="2">
+        <v>121</v>
+      </c>
+      <c r="L14" t="s" s="2">
+        <v>122</v>
+      </c>
+      <c r="M14" t="s" s="2">
+        <v>122</v>
+      </c>
+      <c r="N14" s="2"/>
+      <c r="O14" s="2"/>
+      <c r="P14" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Q14" s="2"/>
+      <c r="R14" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="S14" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="T14" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="U14" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="V14" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="W14" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="X14" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Y14" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Z14" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AA14" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AB14" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AC14" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AD14" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AE14" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AF14" t="s" s="2">
+        <v>120</v>
+      </c>
+      <c r="AG14" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AH14" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AI14" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AJ14" t="s" s="2">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s" s="2">
+        <v>123</v>
+      </c>
+      <c r="B15" t="s" s="2">
+        <v>123</v>
+      </c>
+      <c r="C15" s="2"/>
+      <c r="D15" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="E15" s="2"/>
+      <c r="F15" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="G15" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="H15" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="I15" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="J15" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="K15" t="s" s="2">
+        <v>124</v>
+      </c>
+      <c r="L15" t="s" s="2">
+        <v>125</v>
+      </c>
+      <c r="M15" t="s" s="2">
+        <v>125</v>
+      </c>
+      <c r="N15" s="2"/>
+      <c r="O15" s="2"/>
+      <c r="P15" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Q15" s="2"/>
+      <c r="R15" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="S15" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="T15" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="U15" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="V15" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="W15" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="X15" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Y15" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Z15" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AA15" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AB15" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AC15" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AD15" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AE15" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AF15" t="s" s="2">
+        <v>123</v>
+      </c>
+      <c r="AG15" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH15" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AI15" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AJ15" t="s" s="2">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s" s="2">
+        <v>126</v>
+      </c>
+      <c r="B16" t="s" s="2">
+        <v>126</v>
+      </c>
+      <c r="C16" s="2"/>
+      <c r="D16" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="E16" s="2"/>
+      <c r="F16" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="G16" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="H16" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="I16" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="J16" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="K16" t="s" s="2">
+        <v>127</v>
+      </c>
+      <c r="L16" t="s" s="2">
+        <v>128</v>
+      </c>
+      <c r="M16" t="s" s="2">
+        <v>128</v>
+      </c>
+      <c r="N16" s="2"/>
+      <c r="O16" s="2"/>
+      <c r="P16" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Q16" s="2"/>
+      <c r="R16" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="S16" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="T16" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="U16" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="V16" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="W16" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="X16" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Y16" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Z16" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AA16" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AB16" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AC16" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AD16" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AE16" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AF16" t="s" s="2">
+        <v>126</v>
+      </c>
+      <c r="AG16" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH16" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AI16" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AJ16" t="s" s="2">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s" s="2">
+        <v>129</v>
+      </c>
+      <c r="B17" t="s" s="2">
+        <v>129</v>
+      </c>
+      <c r="C17" s="2"/>
+      <c r="D17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="E17" s="2"/>
+      <c r="F17" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="G17" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="H17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="I17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="J17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="K17" t="s" s="2">
+        <v>130</v>
+      </c>
+      <c r="L17" t="s" s="2">
+        <v>131</v>
+      </c>
+      <c r="M17" t="s" s="2">
+        <v>131</v>
+      </c>
+      <c r="N17" s="2"/>
+      <c r="O17" s="2"/>
+      <c r="P17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Q17" s="2"/>
+      <c r="R17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="S17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="T17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="U17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="V17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="W17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="X17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Y17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="Z17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AA17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AB17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AC17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AD17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AE17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AF17" t="s" s="2">
+        <v>129</v>
+      </c>
+      <c r="AG17" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AH17" t="s" s="2">
+        <v>75</v>
+      </c>
+      <c r="AI17" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AJ17" t="s" s="2">
         <v>73</v>
       </c>
     </row>

</xml_diff>